<commit_message>
Upload full recovery lock cascade package
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step_ru.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step_ru.xlsx
@@ -427,18 +427,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E260"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Поле</t>
+          <t>Field</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Значение</t>
+          <t>Value</t>
         </is>
       </c>
     </row>
@@ -634,12 +634,12 @@
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>БольшойКоэф</t>
+          <t>BigRatio</t>
         </is>
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t>МалыйКоэф</t>
+          <t>SmallRatio</t>
         </is>
       </c>
     </row>
@@ -687,242 +687,6 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -934,23 +698,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E260"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Правило</t>
+          <t>Rule</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>ВВЕРХ</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>ВНИЗ</t>
+          <t>DOWN</t>
         </is>
       </c>
     </row>
@@ -1029,260 +793,6 @@
         <v/>
       </c>
     </row>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1294,7 +804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E260"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1303,265 +813,6 @@
         <v/>
       </c>
     </row>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1573,33 +824,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J260"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Тикет</t>
+          <t>Ticket</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Тип</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Роль</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Лот</t>
+          <t>Lot</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>ЦенаОткрытия</t>
+          <t>OpenPrice</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -1664,6 +915,7 @@
           <t>NO</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1701,6 +953,7 @@
           <t>YES</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1786,261 +1039,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2052,23 +1050,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J260"/>
+  <dimension ref="A1:J225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Поле</t>
+          <t>Field</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Значение</t>
+          <t>Value</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>СредняяЦенаBUY</t>
+          <t>AverageBuyPrice</t>
         </is>
       </c>
       <c r="E1">
@@ -2079,7 +1077,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ТекущаяЦена</t>
+          <t>CurrentPrice</t>
         </is>
       </c>
       <c r="B2">
@@ -2088,7 +1086,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>СредняяЦенаSELL</t>
+          <t>AverageSellPrice</t>
         </is>
       </c>
       <c r="E2">
@@ -2099,7 +1097,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ДвижениеВверхПункты</t>
+          <t>MoveUpPoints</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -2107,7 +1105,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Центр</t>
+          <t>Center</t>
         </is>
       </c>
       <c r="E3">
@@ -2118,7 +1116,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>СценарнаяЦена</t>
+          <t>ScenarioPrice</t>
         </is>
       </c>
       <c r="B4">
@@ -2127,7 +1125,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ВерхУровень1</t>
+          <t>UpperLevel1</t>
         </is>
       </c>
       <c r="E4">
@@ -2138,7 +1136,7 @@
     <row r="5">
       <c r="D5" t="inlineStr">
         <is>
-          <t>ВерхУровень2</t>
+          <t>UpperLevel2</t>
         </is>
       </c>
       <c r="E5">
@@ -2149,22 +1147,22 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Тикет</t>
+          <t>Ticket</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>Тип</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>Роль</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>ВерхУровень3</t>
+          <t>UpperLevel3</t>
         </is>
       </c>
       <c r="E6" s="1">
@@ -2212,7 +1210,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ВерхУровень4</t>
+          <t>UpperLevel4</t>
         </is>
       </c>
       <c r="E7">
@@ -2297,7 +1295,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>НизУровень1</t>
+          <t>LowerLevel1</t>
         </is>
       </c>
       <c r="E9">
@@ -2340,7 +1338,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>НизУровень2</t>
+          <t>LowerLevel2</t>
         </is>
       </c>
       <c r="E10">
@@ -2383,7 +1381,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>НизУровень3</t>
+          <t>LowerLevel3</t>
         </is>
       </c>
       <c r="E11">
@@ -2426,7 +1424,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>НизУровень4</t>
+          <t>LowerLevel4</t>
         </is>
       </c>
       <c r="E12">
@@ -10602,23 +9600,10 @@
         <v/>
       </c>
     </row>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>ТипХвоста</t>
+          <t>TailType</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -10630,7 +9615,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>ХудшийPnLХвоста</t>
+          <t>TailWorstPnL</t>
         </is>
       </c>
       <c r="B221">
@@ -10641,7 +9626,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>ТикетХвоста</t>
+          <t>TailTicket</t>
         </is>
       </c>
       <c r="B222">
@@ -10652,7 +9637,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>ЛотХвоста</t>
+          <t>TailLot</t>
         </is>
       </c>
       <c r="B223">
@@ -10663,7 +9648,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>УбытокХвостаДеньги</t>
+          <t>TailLossMoney</t>
         </is>
       </c>
       <c r="B224">
@@ -10674,7 +9659,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>УбытокНаЛот</t>
+          <t>TailLossPerLot</t>
         </is>
       </c>
       <c r="B225">
@@ -10682,41 +9667,6 @@
         <v/>
       </c>
     </row>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10728,23 +9678,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J260"/>
+  <dimension ref="A1:J225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Поле</t>
+          <t>Field</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Значение</t>
+          <t>Value</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>СредняяЦенаBUY</t>
+          <t>AverageBuyPrice</t>
         </is>
       </c>
       <c r="E1">
@@ -10755,7 +9705,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ТекущаяЦена</t>
+          <t>CurrentPrice</t>
         </is>
       </c>
       <c r="B2">
@@ -10764,7 +9714,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>СредняяЦенаSELL</t>
+          <t>AverageSellPrice</t>
         </is>
       </c>
       <c r="E2">
@@ -10775,7 +9725,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ДвижениеВнизПункты</t>
+          <t>MoveDownPoints</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -10783,7 +9733,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Центр</t>
+          <t>Center</t>
         </is>
       </c>
       <c r="E3">
@@ -10794,7 +9744,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>СценарнаяЦена</t>
+          <t>ScenarioPrice</t>
         </is>
       </c>
       <c r="B4">
@@ -10803,7 +9753,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ВерхУровень1</t>
+          <t>UpperLevel1</t>
         </is>
       </c>
       <c r="E4">
@@ -10814,7 +9764,7 @@
     <row r="5">
       <c r="D5" t="inlineStr">
         <is>
-          <t>ВерхУровень2</t>
+          <t>UpperLevel2</t>
         </is>
       </c>
       <c r="E5">
@@ -10825,22 +9775,22 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Тикет</t>
+          <t>Ticket</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>Тип</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>Роль</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>ВерхУровень3</t>
+          <t>UpperLevel3</t>
         </is>
       </c>
       <c r="E6" s="1">
@@ -10888,7 +9838,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ВерхУровень4</t>
+          <t>UpperLevel4</t>
         </is>
       </c>
       <c r="E7">
@@ -10973,7 +9923,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>НизУровень1</t>
+          <t>LowerLevel1</t>
         </is>
       </c>
       <c r="E9">
@@ -11016,7 +9966,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>НизУровень2</t>
+          <t>LowerLevel2</t>
         </is>
       </c>
       <c r="E10">
@@ -11059,7 +10009,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>НизУровень3</t>
+          <t>LowerLevel3</t>
         </is>
       </c>
       <c r="E11">
@@ -11102,7 +10052,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>НизУровень4</t>
+          <t>LowerLevel4</t>
         </is>
       </c>
       <c r="E12">
@@ -19278,23 +18228,10 @@
         <v/>
       </c>
     </row>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>ТипХвоста</t>
+          <t>TailType</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -19306,7 +18243,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>ХудшийPnLХвоста</t>
+          <t>TailWorstPnL</t>
         </is>
       </c>
       <c r="B221">
@@ -19317,7 +18254,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>ТикетХвоста</t>
+          <t>TailTicket</t>
         </is>
       </c>
       <c r="B222">
@@ -19328,7 +18265,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>ЛотХвоста</t>
+          <t>TailLot</t>
         </is>
       </c>
       <c r="B223">
@@ -19339,7 +18276,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>УбытокХвостаДеньги</t>
+          <t>TailLossMoney</t>
         </is>
       </c>
       <c r="B224">
@@ -19350,7 +18287,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>УбытокНаЛот</t>
+          <t>TailLossPerLot</t>
         </is>
       </c>
       <c r="B225">
@@ -19358,41 +18295,6 @@
         <v/>
       </c>
     </row>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19404,25 +18306,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R260"/>
+  <dimension ref="A1:R36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Поле</t>
+          <t>Field</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Значение</t>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ТипХвоста</t>
+          <t>TailType</t>
         </is>
       </c>
       <c r="B2">
@@ -19433,7 +18335,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ЛотХвоста</t>
+          <t>TailLot</t>
         </is>
       </c>
       <c r="B3">
@@ -19444,7 +18346,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>СледующийУровень</t>
+          <t>NextLevel</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -19454,7 +18356,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>БольшойКоэф</t>
+          <t>BigRatio</t>
         </is>
       </c>
       <c r="B5">
@@ -19465,7 +18367,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>МалыйКоэф</t>
+          <t>SmallRatio</t>
         </is>
       </c>
       <c r="B6">
@@ -19476,7 +18378,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>БольшойЛот</t>
+          <t>BigLot</t>
         </is>
       </c>
       <c r="B7">
@@ -19487,7 +18389,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>МалыйЛот</t>
+          <t>SmallLot</t>
         </is>
       </c>
       <c r="B8">
@@ -19498,7 +18400,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>АктивныеСекции</t>
+          <t>ActiveSections</t>
         </is>
       </c>
       <c r="B9">
@@ -19509,7 +18411,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ОбщийЛотПослеОткрытия</t>
+          <t>TotalLotAfterOpen</t>
         </is>
       </c>
       <c r="B10">
@@ -19520,7 +18422,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ЧистыйЛотПослеОткрытия</t>
+          <t>NetLotAfterOpen</t>
         </is>
       </c>
       <c r="B11">
@@ -19531,7 +18433,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>УровеньДостигнут</t>
+          <t>LevelReached</t>
         </is>
       </c>
       <c r="B12">
@@ -19542,7 +18444,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>НетВстречногоКаскада</t>
+          <t>NoOppositeCascade</t>
         </is>
       </c>
       <c r="B13">
@@ -19553,7 +18455,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>МожноОткрытьСекцию</t>
+          <t>CanOpenSection</t>
         </is>
       </c>
       <c r="B14">
@@ -19561,15 +18463,10 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>IDСекции</t>
+          <t>SectionID</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -19579,7 +18476,7 @@
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t>БольшойЛот</t>
+          <t>BigLot</t>
         </is>
       </c>
       <c r="D20" s="1" t="inlineStr">
@@ -19958,15 +18855,10 @@
         <v/>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ВыбраннаяСекция</t>
+          <t>SelectedSectionID</t>
         </is>
       </c>
       <c r="B30">
@@ -19977,7 +18869,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ПрибыльЦикла</t>
+          <t>CycleProfit</t>
         </is>
       </c>
       <c r="B31">
@@ -19988,7 +18880,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>МожноЗакрытьСекцию</t>
+          <t>CanCloseSection</t>
         </is>
       </c>
       <c r="B32">
@@ -19999,7 +18891,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ДобавкаРезерв</t>
+          <t>ReserveAdd</t>
         </is>
       </c>
       <c r="B33">
@@ -20010,7 +18902,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ДобавкаRecovery</t>
+          <t>RecoveryAdd</t>
         </is>
       </c>
       <c r="B34">
@@ -20021,7 +18913,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>НовыйГлобРезерв</t>
+          <t>NewGlobalReserve</t>
         </is>
       </c>
       <c r="B35">
@@ -20032,7 +18924,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>НовыйRecoveryFund</t>
+          <t>NewRecoveryFund</t>
         </is>
       </c>
       <c r="B36">
@@ -20040,230 +18932,6 @@
         <v/>
       </c>
     </row>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -20275,25 +18943,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R260"/>
+  <dimension ref="A1:R36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Поле</t>
+          <t>Field</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Значение</t>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ТипХвоста</t>
+          <t>TailType</t>
         </is>
       </c>
       <c r="B2">
@@ -20304,7 +18972,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ЛотХвоста</t>
+          <t>TailLot</t>
         </is>
       </c>
       <c r="B3">
@@ -20315,7 +18983,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>СледующийУровень</t>
+          <t>NextLevel</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -20325,7 +18993,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>БольшойКоэф</t>
+          <t>BigRatio</t>
         </is>
       </c>
       <c r="B5">
@@ -20336,7 +19004,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>МалыйКоэф</t>
+          <t>SmallRatio</t>
         </is>
       </c>
       <c r="B6">
@@ -20347,7 +19015,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>БольшойЛот</t>
+          <t>BigLot</t>
         </is>
       </c>
       <c r="B7">
@@ -20358,7 +19026,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>МалыйЛот</t>
+          <t>SmallLot</t>
         </is>
       </c>
       <c r="B8">
@@ -20369,7 +19037,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>АктивныеСекции</t>
+          <t>ActiveSections</t>
         </is>
       </c>
       <c r="B9">
@@ -20380,7 +19048,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ОбщийЛотПослеОткрытия</t>
+          <t>TotalLotAfterOpen</t>
         </is>
       </c>
       <c r="B10">
@@ -20391,7 +19059,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ЧистыйЛотПослеОткрытия</t>
+          <t>NetLotAfterOpen</t>
         </is>
       </c>
       <c r="B11">
@@ -20402,7 +19070,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>УровеньДостигнут</t>
+          <t>LevelReached</t>
         </is>
       </c>
       <c r="B12">
@@ -20413,7 +19081,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>НетВстречногоКаскада</t>
+          <t>NoOppositeCascade</t>
         </is>
       </c>
       <c r="B13">
@@ -20424,7 +19092,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>МожноОткрытьСекцию</t>
+          <t>CanOpenSection</t>
         </is>
       </c>
       <c r="B14">
@@ -20432,15 +19100,10 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>IDСекции</t>
+          <t>SectionID</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -20450,7 +19113,7 @@
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t>БольшойЛот</t>
+          <t>BigLot</t>
         </is>
       </c>
       <c r="D20" s="1" t="inlineStr">
@@ -20829,15 +19492,10 @@
         <v/>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ВыбраннаяСекция</t>
+          <t>SelectedSectionID</t>
         </is>
       </c>
       <c r="B30">
@@ -20848,7 +19506,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ПрибыльЦикла</t>
+          <t>CycleProfit</t>
         </is>
       </c>
       <c r="B31">
@@ -20859,7 +19517,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>МожноЗакрытьСекцию</t>
+          <t>CanCloseSection</t>
         </is>
       </c>
       <c r="B32">
@@ -20870,7 +19528,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ДобавкаРезерв</t>
+          <t>ReserveAdd</t>
         </is>
       </c>
       <c r="B33">
@@ -20881,7 +19539,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ДобавкаRecovery</t>
+          <t>RecoveryAdd</t>
         </is>
       </c>
       <c r="B34">
@@ -20892,7 +19550,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>НовыйГлобРезерв</t>
+          <t>NewGlobalReserve</t>
         </is>
       </c>
       <c r="B35">
@@ -20903,7 +19561,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>НовыйRecoveryFund</t>
+          <t>NewRecoveryFund</t>
         </is>
       </c>
       <c r="B36">
@@ -20911,230 +19569,6 @@
         <v/>
       </c>
     </row>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21146,25 +19580,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E260"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Поле</t>
+          <t>Field</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Значение</t>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ТипХвоста</t>
+          <t>TailType</t>
         </is>
       </c>
       <c r="B2">
@@ -21175,7 +19609,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ТикетХвоста</t>
+          <t>TailTicket</t>
         </is>
       </c>
       <c r="B3">
@@ -21186,7 +19620,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ЛотХвоста</t>
+          <t>TailLot</t>
         </is>
       </c>
       <c r="B4">
@@ -21197,7 +19631,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>УбытокНаЛот</t>
+          <t>TailLossPerLot</t>
         </is>
       </c>
       <c r="B5">
@@ -21208,7 +19642,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>МожноЗакрытьСекцию</t>
+          <t>CanCloseSection</t>
         </is>
       </c>
       <c r="B6">
@@ -21219,7 +19653,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RecoveryПослеЦикла</t>
+          <t>RecoveryFundAfterCycle</t>
         </is>
       </c>
       <c r="B7">
@@ -21230,7 +19664,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ЛотЗакрытияСырой</t>
+          <t>CloseLotRaw</t>
         </is>
       </c>
       <c r="B8">
@@ -21241,7 +19675,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ЛотЗакрытияОкругл</t>
+          <t>CloseLotRounded</t>
         </is>
       </c>
       <c r="B9">
@@ -21252,7 +19686,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ЛотЗакрытияФинал</t>
+          <t>CloseLotFinal</t>
         </is>
       </c>
       <c r="B10">
@@ -21263,7 +19697,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ЗакрытиеРазрешено</t>
+          <t>CloseAllowed</t>
         </is>
       </c>
       <c r="B11">
@@ -21274,7 +19708,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>УбытокЗакрытияХвоста</t>
+          <t>TailCloseLoss</t>
         </is>
       </c>
       <c r="B12">
@@ -21285,7 +19719,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RecoveryПослеЗакрытия</t>
+          <t>RecoveryFundAfterClose</t>
         </is>
       </c>
       <c r="B13">
@@ -21296,7 +19730,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ЛотХвостаПослеЗакрытия</t>
+          <t>TailLotAfterClose</t>
         </is>
       </c>
       <c r="B14">
@@ -21307,7 +19741,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>СледующийУровень</t>
+          <t>NextLevel</t>
         </is>
       </c>
       <c r="B15">
@@ -21318,7 +19752,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>СледБольшойЛотПослеRecovery</t>
+          <t>NextBigLotAfterRecovery</t>
         </is>
       </c>
       <c r="B16">
@@ -21329,7 +19763,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>СледМалыйЛотПослеRecovery</t>
+          <t>NextSmallLotAfterRecovery</t>
         </is>
       </c>
       <c r="B17">
@@ -21337,249 +19771,6 @@
         <v/>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21591,25 +19782,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E260"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Поле</t>
+          <t>Field</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Значение</t>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ТипХвоста</t>
+          <t>TailType</t>
         </is>
       </c>
       <c r="B2">
@@ -21620,7 +19811,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ТикетХвоста</t>
+          <t>TailTicket</t>
         </is>
       </c>
       <c r="B3">
@@ -21631,7 +19822,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ЛотХвоста</t>
+          <t>TailLot</t>
         </is>
       </c>
       <c r="B4">
@@ -21642,7 +19833,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>УбытокНаЛот</t>
+          <t>TailLossPerLot</t>
         </is>
       </c>
       <c r="B5">
@@ -21653,7 +19844,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>МожноЗакрытьСекцию</t>
+          <t>CanCloseSection</t>
         </is>
       </c>
       <c r="B6">
@@ -21664,7 +19855,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RecoveryПослеЦикла</t>
+          <t>RecoveryFundAfterCycle</t>
         </is>
       </c>
       <c r="B7">
@@ -21675,7 +19866,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ЛотЗакрытияСырой</t>
+          <t>CloseLotRaw</t>
         </is>
       </c>
       <c r="B8">
@@ -21686,7 +19877,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ЛотЗакрытияОкругл</t>
+          <t>CloseLotRounded</t>
         </is>
       </c>
       <c r="B9">
@@ -21697,7 +19888,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ЛотЗакрытияФинал</t>
+          <t>CloseLotFinal</t>
         </is>
       </c>
       <c r="B10">
@@ -21708,7 +19899,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ЗакрытиеРазрешено</t>
+          <t>CloseAllowed</t>
         </is>
       </c>
       <c r="B11">
@@ -21719,7 +19910,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>УбытокЗакрытияХвоста</t>
+          <t>TailCloseLoss</t>
         </is>
       </c>
       <c r="B12">
@@ -21730,7 +19921,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RecoveryПослеЗакрытия</t>
+          <t>RecoveryFundAfterClose</t>
         </is>
       </c>
       <c r="B13">
@@ -21741,7 +19932,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ЛотХвостаПослеЗакрытия</t>
+          <t>TailLotAfterClose</t>
         </is>
       </c>
       <c r="B14">
@@ -21752,7 +19943,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>СледующийУровень</t>
+          <t>NextLevel</t>
         </is>
       </c>
       <c r="B15">
@@ -21763,7 +19954,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>СледБольшойЛотПослеRecovery</t>
+          <t>NextBigLotAfterRecovery</t>
         </is>
       </c>
       <c r="B16">
@@ -21774,7 +19965,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>СледМалыйЛотПослеRecovery</t>
+          <t>NextSmallLotAfterRecovery</t>
         </is>
       </c>
       <c r="B17">
@@ -21782,249 +19973,6 @@
         <v/>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -22036,30 +19984,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E260"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Поле</t>
+          <t>Field</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>ВВЕРХ</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>ВНИЗ</t>
+          <t>DOWN</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>СценарнаяЦена</t>
+          <t>ScenarioPrice</t>
         </is>
       </c>
       <c r="B2">
@@ -22074,7 +20022,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ПлавающийИтогКорзины</t>
+          <t>BasketFloating</t>
         </is>
       </c>
       <c r="B3">
@@ -22089,7 +20037,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ГлобРезервПосле</t>
+          <t>GlobalReserveAfter</t>
         </is>
       </c>
       <c r="B4">
@@ -22104,7 +20052,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>RecoveryПослеЦикла</t>
+          <t>RecoveryFundAfterCycle</t>
         </is>
       </c>
       <c r="B5">
@@ -22119,7 +20067,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ЛотХвостаПосле</t>
+          <t>TailLotAfter</t>
         </is>
       </c>
       <c r="B6">
@@ -22134,7 +20082,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ЛотЗакрытия</t>
+          <t>CloseLot</t>
         </is>
       </c>
       <c r="B7">
@@ -22149,7 +20097,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>МожноЗакрытьСекцию</t>
+          <t>CanCloseSection</t>
         </is>
       </c>
       <c r="B8">
@@ -22164,7 +20112,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>МожноЗакрытьХвост</t>
+          <t>CanCloseTail</t>
         </is>
       </c>
       <c r="B9">
@@ -22179,7 +20127,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>МожноЗакрытьКорзину</t>
+          <t>CanCloseBasket</t>
         </is>
       </c>
       <c r="B10">
@@ -22194,7 +20142,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>СледБольшойЛот</t>
+          <t>NextBigLot</t>
         </is>
       </c>
       <c r="B11">
@@ -22209,7 +20157,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>СледМалыйЛот</t>
+          <t>NextSmallLot</t>
         </is>
       </c>
       <c r="B12">
@@ -22224,7 +20172,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>СледДействие</t>
+          <t>NextAction</t>
         </is>
       </c>
       <c r="B13">
@@ -22236,253 +20184,6 @@
         <v/>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>